<commit_message>
Price Full Detail by vehicle ($215/$250/$300), compare sub vs tech pay
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XeYkWCpV7g2ezgB3AXjkpD
</commit_message>
<xml_diff>
--- a/Coastline_Price_Sheet.xlsx
+++ b/Coastline_Price_Sheet.xlsx
@@ -423,10 +423,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F38"/>
+  <dimension ref="A1:J38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="48" customWidth="1" min="1" max="1"/>
+    <col width="46" customWidth="1" min="1" max="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -446,7 +446,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>One service, one price. Yellow cells are yours to change. Updated Oct 26, 2026.</t>
+          <t>Full Detail only, priced by vehicle. No packages. Yellow cells are yours to change. Updated Oct 26, 2026.</t>
         </is>
       </c>
     </row>
@@ -465,443 +465,501 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Full Detail price</t>
+          <t>Rapid Reach fee per job (off the top)</t>
         </is>
       </c>
       <c r="B6" s="2" t="n">
-        <v>315</v>
+        <v>25</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Rapid Reach fee per job (off the top)</t>
+          <t>Subcontractor share (after fee)</t>
         </is>
       </c>
       <c r="B7" s="2" t="n">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>Subcontractor share</t>
-        </is>
-      </c>
-      <c r="B8" s="2" t="n">
         <v>0.6</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>Morgan share</t>
-        </is>
-      </c>
-      <c r="B9">
-        <f>1-B8</f>
+      <c r="A9" s="1" t="inlineStr">
+        <is>
+          <t>Vehicle</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Price</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Rapid Reach</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>SUBCONTRACTOR: Sub gets (60%)</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Morgan keeps</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Margin</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>TECH PAY: Tech pay</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Supplies</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>Morgan keeps</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>Margin</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Sedan</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="n">
+        <v>215</v>
+      </c>
+      <c r="C10">
+        <f>$B$6</f>
+        <v/>
+      </c>
+      <c r="D10">
+        <f>ROUND((B10-C10)*$B$7,2)</f>
+        <v/>
+      </c>
+      <c r="E10">
+        <f>B10-C10-D10</f>
+        <v/>
+      </c>
+      <c r="F10">
+        <f>E10/B10</f>
+        <v/>
+      </c>
+      <c r="G10" s="2" t="n">
+        <v>70</v>
+      </c>
+      <c r="H10" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="I10">
+        <f>B10-C10-G10-H10</f>
+        <v/>
+      </c>
+      <c r="J10">
+        <f>I10/B10</f>
         <v/>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="1" t="inlineStr">
-        <is>
-          <t>PER JOB</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>Amount</t>
-        </is>
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>SUV</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="n">
+        <v>250</v>
+      </c>
+      <c r="C11">
+        <f>$B$6</f>
+        <v/>
+      </c>
+      <c r="D11">
+        <f>ROUND((B11-C11)*$B$7,2)</f>
+        <v/>
+      </c>
+      <c r="E11">
+        <f>B11-C11-D11</f>
+        <v/>
+      </c>
+      <c r="F11">
+        <f>E11/B11</f>
+        <v/>
+      </c>
+      <c r="G11" s="2" t="n">
+        <v>70</v>
+      </c>
+      <c r="H11" s="2" t="n">
+        <v>18</v>
+      </c>
+      <c r="I11">
+        <f>B11-C11-G11-H11</f>
+        <v/>
+      </c>
+      <c r="J11">
+        <f>I11/B11</f>
+        <v/>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Customer pays</t>
-        </is>
-      </c>
-      <c r="B12">
-        <f>B6</f>
-        <v/>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>Rapid Reach fee</t>
-        </is>
-      </c>
-      <c r="B13">
-        <f>-B7</f>
+          <t>Truck</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="n">
+        <v>300</v>
+      </c>
+      <c r="C12">
+        <f>$B$6</f>
+        <v/>
+      </c>
+      <c r="D12">
+        <f>ROUND((B12-C12)*$B$7,2)</f>
+        <v/>
+      </c>
+      <c r="E12">
+        <f>B12-C12-D12</f>
+        <v/>
+      </c>
+      <c r="F12">
+        <f>E12/B12</f>
+        <v/>
+      </c>
+      <c r="G12" s="2" t="n">
+        <v>70</v>
+      </c>
+      <c r="H12" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="I12">
+        <f>B12-C12-G12-H12</f>
+        <v/>
+      </c>
+      <c r="J12">
+        <f>I12/B12</f>
         <v/>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Left to split</t>
+          <t>Avg ticket (40% sedan / 40% SUV / 20% truck)</t>
         </is>
       </c>
       <c r="B14">
-        <f>B6-B7</f>
+        <f>0.4*B10+0.4*B11+0.2*B12</f>
         <v/>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Subcontractor (60%)</t>
+          <t>Avg Morgan keeps per job: subcontractors</t>
         </is>
       </c>
       <c r="B15">
-        <f>ROUND(B14*B8,2)</f>
+        <f>0.4*E10+0.4*E11+0.2*E12</f>
         <v/>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Morgan keeps (40%)</t>
+          <t>Avg Morgan keeps per job: tech pay</t>
         </is>
       </c>
       <c r="B16">
-        <f>ROUND(B14*B9,2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>Morgan margin (of price)</t>
-        </is>
-      </c>
-      <c r="B17">
-        <f>B16/B6</f>
-        <v/>
+        <f>0.4*I10+0.4*I11+0.2*I12</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="1" t="inlineStr">
+        <is>
+          <t>Monthly revenue</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Jobs</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Morgan keeps (subcontractors)</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Morgan keeps (tech pay)</t>
+        </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="1" t="inlineStr">
-        <is>
-          <t>MONTHLY</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>Revenue</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>Jobs</t>
-        </is>
-      </c>
-      <c r="D19" t="inlineStr">
-        <is>
-          <t>Paid to subs</t>
-        </is>
-      </c>
-      <c r="E19" t="inlineStr">
-        <is>
-          <t>Rapid Reach</t>
-        </is>
-      </c>
-      <c r="F19" t="inlineStr">
-        <is>
-          <t>Morgan keeps</t>
-        </is>
+      <c r="A19" t="n">
+        <v>10000</v>
+      </c>
+      <c r="B19">
+        <f>ROUNDUP(A19/$B$14,0)</f>
+        <v/>
+      </c>
+      <c r="C19">
+        <f>ROUND(B19*$B$15,0)</f>
+        <v/>
+      </c>
+      <c r="D19">
+        <f>ROUND(B19*$B$16,0)</f>
+        <v/>
       </c>
     </row>
     <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>$10,000 month</t>
-        </is>
-      </c>
-      <c r="B20" t="n">
-        <v>10000</v>
+      <c r="A20" t="n">
+        <v>20000</v>
+      </c>
+      <c r="B20">
+        <f>ROUNDUP(A20/$B$14,0)</f>
+        <v/>
       </c>
       <c r="C20">
-        <f>ROUNDUP(B20/$B$6,0)</f>
+        <f>ROUND(B20*$B$15,0)</f>
         <v/>
       </c>
       <c r="D20">
-        <f>C20*$B$15</f>
-        <v/>
-      </c>
-      <c r="E20">
-        <f>C20*$B$7</f>
-        <v/>
-      </c>
-      <c r="F20">
-        <f>C20*$B$16</f>
+        <f>ROUND(B20*$B$16,0)</f>
         <v/>
       </c>
     </row>
     <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>$20,000 month</t>
-        </is>
-      </c>
-      <c r="B21" t="n">
-        <v>20000</v>
+      <c r="A21" t="n">
+        <v>30000</v>
+      </c>
+      <c r="B21">
+        <f>ROUNDUP(A21/$B$14,0)</f>
+        <v/>
       </c>
       <c r="C21">
-        <f>ROUNDUP(B21/$B$6,0)</f>
+        <f>ROUND(B21*$B$15,0)</f>
         <v/>
       </c>
       <c r="D21">
-        <f>C21*$B$15</f>
-        <v/>
-      </c>
-      <c r="E21">
-        <f>C21*$B$7</f>
-        <v/>
-      </c>
-      <c r="F21">
-        <f>C21*$B$16</f>
+        <f>ROUND(B21*$B$16,0)</f>
         <v/>
       </c>
     </row>
     <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>$30,000 month</t>
-        </is>
-      </c>
-      <c r="B22" t="n">
-        <v>30000</v>
+      <c r="A22" t="n">
+        <v>50000</v>
+      </c>
+      <c r="B22">
+        <f>ROUNDUP(A22/$B$14,0)</f>
+        <v/>
       </c>
       <c r="C22">
-        <f>ROUNDUP(B22/$B$6,0)</f>
+        <f>ROUND(B22*$B$15,0)</f>
         <v/>
       </c>
       <c r="D22">
-        <f>C22*$B$15</f>
-        <v/>
-      </c>
-      <c r="E22">
-        <f>C22*$B$7</f>
-        <v/>
-      </c>
-      <c r="F22">
-        <f>C22*$B$16</f>
+        <f>ROUND(B22*$B$16,0)</f>
         <v/>
       </c>
     </row>
     <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>$50,000 month</t>
-        </is>
-      </c>
-      <c r="B23" t="n">
-        <v>50000</v>
+      <c r="A23" t="n">
+        <v>100000</v>
+      </c>
+      <c r="B23">
+        <f>ROUNDUP(A23/$B$14,0)</f>
+        <v/>
       </c>
       <c r="C23">
-        <f>ROUNDUP(B23/$B$6,0)</f>
+        <f>ROUND(B23*$B$15,0)</f>
         <v/>
       </c>
       <c r="D23">
-        <f>C23*$B$15</f>
-        <v/>
-      </c>
-      <c r="E23">
-        <f>C23*$B$7</f>
-        <v/>
-      </c>
-      <c r="F23">
-        <f>C23*$B$16</f>
-        <v/>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>$100,000 month</t>
-        </is>
-      </c>
-      <c r="B24" t="n">
-        <v>100000</v>
-      </c>
-      <c r="C24">
-        <f>ROUNDUP(B24/$B$6,0)</f>
-        <v/>
-      </c>
-      <c r="D24">
-        <f>C24*$B$15</f>
-        <v/>
-      </c>
-      <c r="E24">
-        <f>C24*$B$7</f>
-        <v/>
-      </c>
-      <c r="F24">
-        <f>C24*$B$16</f>
-        <v/>
+        <f>ROUND(B23*$B$16,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="1" t="inlineStr">
+        <is>
+          <t>EXTRAS (only if the car needs it; no Rapid Reach fee)</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Price</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Sub (60%)</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Morgan (40%)</t>
+        </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>EXTRAS (only if the car needs it; no Rapid Reach fee)</t>
-        </is>
-      </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>Price</t>
-        </is>
-      </c>
-      <c r="C26" t="inlineStr">
-        <is>
-          <t>Sub (60%)</t>
-        </is>
-      </c>
-      <c r="D26" t="inlineStr">
-        <is>
-          <t>Morgan (40%)</t>
-        </is>
+          <t>Heavy pet hair</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>50</v>
+      </c>
+      <c r="C26">
+        <f>B26*$B$7</f>
+        <v/>
+      </c>
+      <c r="D26">
+        <f>B26*(1-$B$7)</f>
+        <v/>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Heavy pet hair</t>
+          <t>Odor removal (ozone)</t>
         </is>
       </c>
       <c r="B27" t="n">
-        <v>50</v>
+        <v>75</v>
       </c>
       <c r="C27">
-        <f>B27*$B$8</f>
+        <f>B27*$B$7</f>
         <v/>
       </c>
       <c r="D27">
-        <f>B27*$B$9</f>
+        <f>B27*(1-$B$7)</f>
         <v/>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Odor removal (ozone)</t>
+          <t>Headlight restoration</t>
         </is>
       </c>
       <c r="B28" t="n">
         <v>75</v>
       </c>
       <c r="C28">
-        <f>B28*$B$8</f>
+        <f>B28*$B$7</f>
         <v/>
       </c>
       <c r="D28">
-        <f>B28*$B$9</f>
+        <f>B28*(1-$B$7)</f>
         <v/>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Headlight restoration</t>
+          <t>Clay bar + paint sealant (6 months)</t>
         </is>
       </c>
       <c r="B29" t="n">
-        <v>75</v>
+        <v>99</v>
       </c>
       <c r="C29">
-        <f>B29*$B$8</f>
+        <f>B29*$B$7</f>
         <v/>
       </c>
       <c r="D29">
-        <f>B29*$B$9</f>
+        <f>B29*(1-$B$7)</f>
         <v/>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Clay bar + paint sealant (6 months)</t>
+          <t>Heavy dirt / sand / mud</t>
         </is>
       </c>
       <c r="B30" t="n">
-        <v>99</v>
+        <v>50</v>
       </c>
       <c r="C30">
-        <f>B30*$B$8</f>
+        <f>B30*$B$7</f>
         <v/>
       </c>
       <c r="D30">
-        <f>B30*$B$9</f>
+        <f>B30*(1-$B$7)</f>
         <v/>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Heavy dirt / sand / mud</t>
+          <t>Biohazard (from)</t>
         </is>
       </c>
       <c r="B31" t="n">
-        <v>50</v>
+        <v>150</v>
       </c>
       <c r="C31">
-        <f>B31*$B$8</f>
+        <f>B31*$B$7</f>
         <v/>
       </c>
       <c r="D31">
-        <f>B31*$B$9</f>
+        <f>B31*(1-$B$7)</f>
         <v/>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Biohazard (from)</t>
+          <t>Travel (45+ min)</t>
         </is>
       </c>
       <c r="B32" t="n">
-        <v>150</v>
+        <v>35</v>
       </c>
       <c r="C32">
-        <f>B32*$B$8</f>
+        <f>B32*$B$7</f>
         <v/>
       </c>
       <c r="D32">
-        <f>B32*$B$9</f>
-        <v/>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t>Travel (45+ min)</t>
-        </is>
-      </c>
-      <c r="B33" t="n">
-        <v>35</v>
-      </c>
-      <c r="C33">
-        <f>B33*$B$8</f>
-        <v/>
-      </c>
-      <c r="D33">
-        <f>B33*$B$9</f>
-        <v/>
+        <f>B32*(1-$B$7)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="1" t="inlineStr">
+        <is>
+          <t>PRICE RULES</t>
+        </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>PRICE RULES</t>
+          <t>Full Detail only: Sedan $215, SUV $250, Truck $300. No packages.</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>One price: $315 Full Detail. No packages.</t>
+          <t>Always ask the year, make and model before quoting.</t>
         </is>
       </c>
     </row>
@@ -915,7 +973,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Raise prices 5–10% a year with 30 days' notice.</t>
+          <t>Tech pay model: Morgan buys supplies. Subcontractor model: subs pay their own chemicals and gas.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Set Full Detail prices to $234/$285/$325, add on-site add-on rules
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XeYkWCpV7g2ezgB3AXjkpD
</commit_message>
<xml_diff>
--- a/Coastline_Price_Sheet.xlsx
+++ b/Coastline_Price_Sheet.xlsx
@@ -423,7 +423,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J38"/>
+  <dimension ref="A1:J44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -541,7 +541,7 @@
         </is>
       </c>
       <c r="B10" s="2" t="n">
-        <v>215</v>
+        <v>234</v>
       </c>
       <c r="C10">
         <f>$B$6</f>
@@ -581,7 +581,7 @@
         </is>
       </c>
       <c r="B11" s="2" t="n">
-        <v>250</v>
+        <v>285</v>
       </c>
       <c r="C11">
         <f>$B$6</f>
@@ -621,7 +621,7 @@
         </is>
       </c>
       <c r="B12" s="2" t="n">
-        <v>300</v>
+        <v>325</v>
       </c>
       <c r="C12">
         <f>$B$6</f>
@@ -797,7 +797,7 @@
     <row r="25">
       <c r="A25" s="1" t="inlineStr">
         <is>
-          <t>EXTRAS (only if the car needs it; no Rapid Reach fee)</t>
+          <t>ADD-ONS (no Rapid Reach fee; get a yes before starting)</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -819,7 +819,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Heavy pet hair</t>
+          <t>Pet hair removal</t>
         </is>
       </c>
       <c r="B26" t="n">
@@ -837,11 +837,11 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Odor removal (ozone)</t>
+          <t>Heavy pet hair</t>
         </is>
       </c>
       <c r="B27" t="n">
-        <v>75</v>
+        <v>100</v>
       </c>
       <c r="C27">
         <f>B27*$B$7</f>
@@ -855,11 +855,11 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Headlight restoration</t>
+          <t>Seat / stain extraction (per seat)</t>
         </is>
       </c>
       <c r="B28" t="n">
-        <v>75</v>
+        <v>40</v>
       </c>
       <c r="C28">
         <f>B28*$B$7</f>
@@ -873,11 +873,11 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Clay bar + paint sealant (6 months)</t>
+          <t>Carpet + mat shampoo</t>
         </is>
       </c>
       <c r="B29" t="n">
-        <v>99</v>
+        <v>75</v>
       </c>
       <c r="C29">
         <f>B29*$B$7</f>
@@ -891,11 +891,11 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Heavy dirt / sand / mud</t>
+          <t>Odor removal (ozone)</t>
         </is>
       </c>
       <c r="B30" t="n">
-        <v>50</v>
+        <v>75</v>
       </c>
       <c r="C30">
         <f>B30*$B$7</f>
@@ -909,11 +909,11 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Biohazard (from)</t>
+          <t>Headlight restoration</t>
         </is>
       </c>
       <c r="B31" t="n">
-        <v>150</v>
+        <v>75</v>
       </c>
       <c r="C31">
         <f>B31*$B$7</f>
@@ -927,11 +927,11 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Travel (45+ min)</t>
+          <t>Engine bay clean</t>
         </is>
       </c>
       <c r="B32" t="n">
-        <v>35</v>
+        <v>50</v>
       </c>
       <c r="C32">
         <f>B32*$B$7</f>
@@ -942,36 +942,122 @@
         <v/>
       </c>
     </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Clay bar + paint sealant (6 months)</t>
+        </is>
+      </c>
+      <c r="B33" t="n">
+        <v>99</v>
+      </c>
+      <c r="C33">
+        <f>B33*$B$7</f>
+        <v/>
+      </c>
+      <c r="D33">
+        <f>B33*(1-$B$7)</f>
+        <v/>
+      </c>
+    </row>
     <row r="34">
-      <c r="A34" s="1" t="inlineStr">
-        <is>
-          <t>PRICE RULES</t>
-        </is>
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Heavy dirt / sand / mud</t>
+        </is>
+      </c>
+      <c r="B34" t="n">
+        <v>50</v>
+      </c>
+      <c r="C34">
+        <f>B34*$B$7</f>
+        <v/>
+      </c>
+      <c r="D34">
+        <f>B34*(1-$B$7)</f>
+        <v/>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Full Detail only: Sedan $215, SUV $250, Truck $300. No packages.</t>
-        </is>
+          <t>Biohazard (from)</t>
+        </is>
+      </c>
+      <c r="B35" t="n">
+        <v>150</v>
+      </c>
+      <c r="C35">
+        <f>B35*$B$7</f>
+        <v/>
+      </c>
+      <c r="D35">
+        <f>B35*(1-$B$7)</f>
+        <v/>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
+          <t>Travel (45+ min)</t>
+        </is>
+      </c>
+      <c r="B36" t="n">
+        <v>35</v>
+      </c>
+      <c r="C36">
+        <f>B36*$B$7</f>
+        <v/>
+      </c>
+      <c r="D36">
+        <f>B36*(1-$B$7)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="1" t="inlineStr">
+        <is>
+          <t>PRICE RULES</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>Full Detail only: Sedan $234, SUV $285, Truck $325. No packages.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
           <t>Always ask the year, make and model before quoting.</t>
         </is>
       </c>
     </row>
-    <row r="37">
-      <c r="A37" t="inlineStr">
-        <is>
-          <t>Never discount. Heavy pet hair, dirt or biohazard is quoted before the job, never after.</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" t="inlineStr">
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>On the call: mention pet hair / stains / smell add-on prices if the customer brings them up.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>On site: walk around with the customer, point out what you see, quote the add-on from this list, get a yes (text is fine) BEFORE starting.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Never add a charge after the job. Never invent prices on the spot; only use this list.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
         <is>
           <t>Tech pay model: Morgan buys supplies. Subcontractor model: subs pay their own chemicals and gas.</t>
         </is>

</xml_diff>

<commit_message>
Switch to Standard and Luxury packages, update Drive links
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XeYkWCpV7g2ezgB3AXjkpD
</commit_message>
<xml_diff>
--- a/Coastline_Price_Sheet.xlsx
+++ b/Coastline_Price_Sheet.xlsx
@@ -423,10 +423,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J44"/>
+  <dimension ref="A1:H45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="46" customWidth="1" min="1" max="1"/>
+    <col width="40" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -446,7 +447,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Full Detail only, priced by vehicle. No packages. Yellow cells are yours to change. Updated Oct 26, 2026.</t>
+          <t>Two packages: Standard and Luxury. Yellow cells are yours to change. Updated Oct 31, 2026.</t>
         </is>
       </c>
     </row>
@@ -485,449 +486,410 @@
     <row r="9">
       <c r="A9" s="1" t="inlineStr">
         <is>
+          <t>Package</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
           <t>Vehicle</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr">
+      <c r="C9" t="inlineStr">
         <is>
           <t>Price</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr">
+      <c r="D9" t="inlineStr">
         <is>
           <t>Rapid Reach</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>SUBCONTRACTOR: Sub gets (60%)</t>
-        </is>
-      </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Morgan keeps</t>
+          <t>Sub gets (60%)</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
+          <t>You keep (40%)</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
           <t>Margin</t>
         </is>
       </c>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>TECH PAY: Tech pay</t>
-        </is>
-      </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>Supplies</t>
-        </is>
-      </c>
-      <c r="I9" t="inlineStr">
-        <is>
-          <t>Morgan keeps</t>
-        </is>
-      </c>
-      <c r="J9" t="inlineStr">
-        <is>
-          <t>Margin</t>
+          <t>Job mix</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
           <t>Sedan</t>
         </is>
       </c>
-      <c r="B10" s="2" t="n">
-        <v>234</v>
-      </c>
-      <c r="C10">
+      <c r="C10" s="2" t="n">
+        <v>225</v>
+      </c>
+      <c r="D10">
         <f>$B$6</f>
         <v/>
       </c>
-      <c r="D10">
-        <f>ROUND((B10-C10)*$B$7,2)</f>
-        <v/>
-      </c>
       <c r="E10">
-        <f>B10-C10-D10</f>
+        <f>ROUND((C10-D10)*$B$7,2)</f>
         <v/>
       </c>
       <c r="F10">
-        <f>E10/B10</f>
-        <v/>
-      </c>
-      <c r="G10" s="2" t="n">
-        <v>70</v>
+        <f>C10-D10-E10</f>
+        <v/>
+      </c>
+      <c r="G10">
+        <f>F10/C10</f>
+        <v/>
       </c>
       <c r="H10" s="2" t="n">
-        <v>15</v>
-      </c>
-      <c r="I10">
-        <f>B10-C10-G10-H10</f>
-        <v/>
-      </c>
-      <c r="J10">
-        <f>I10/B10</f>
-        <v/>
+        <v>0.28</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
           <t>SUV</t>
         </is>
       </c>
-      <c r="B11" s="2" t="n">
-        <v>285</v>
-      </c>
-      <c r="C11">
+      <c r="C11" s="2" t="n">
+        <v>250</v>
+      </c>
+      <c r="D11">
         <f>$B$6</f>
         <v/>
       </c>
-      <c r="D11">
-        <f>ROUND((B11-C11)*$B$7,2)</f>
-        <v/>
-      </c>
       <c r="E11">
-        <f>B11-C11-D11</f>
+        <f>ROUND((C11-D11)*$B$7,2)</f>
         <v/>
       </c>
       <c r="F11">
-        <f>E11/B11</f>
-        <v/>
-      </c>
-      <c r="G11" s="2" t="n">
-        <v>70</v>
+        <f>C11-D11-E11</f>
+        <v/>
+      </c>
+      <c r="G11">
+        <f>F11/C11</f>
+        <v/>
       </c>
       <c r="H11" s="2" t="n">
-        <v>18</v>
-      </c>
-      <c r="I11">
-        <f>B11-C11-G11-H11</f>
-        <v/>
-      </c>
-      <c r="J11">
-        <f>I11/B11</f>
-        <v/>
+        <v>0.28</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Truck</t>
-        </is>
-      </c>
-      <c r="B12" s="2" t="n">
-        <v>325</v>
-      </c>
-      <c r="C12">
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Truck / 3-row</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="n">
+        <v>275</v>
+      </c>
+      <c r="D12">
         <f>$B$6</f>
         <v/>
       </c>
-      <c r="D12">
-        <f>ROUND((B12-C12)*$B$7,2)</f>
-        <v/>
-      </c>
       <c r="E12">
-        <f>B12-C12-D12</f>
+        <f>ROUND((C12-D12)*$B$7,2)</f>
         <v/>
       </c>
       <c r="F12">
-        <f>E12/B12</f>
-        <v/>
-      </c>
-      <c r="G12" s="2" t="n">
-        <v>70</v>
+        <f>C12-D12-E12</f>
+        <v/>
+      </c>
+      <c r="G12">
+        <f>F12/C12</f>
+        <v/>
       </c>
       <c r="H12" s="2" t="n">
-        <v>20</v>
-      </c>
-      <c r="I12">
-        <f>B12-C12-G12-H12</f>
-        <v/>
-      </c>
-      <c r="J12">
-        <f>I12/B12</f>
-        <v/>
+        <v>0.14</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Luxury</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Sedan</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="n">
+        <v>349</v>
+      </c>
+      <c r="D13">
+        <f>$B$6</f>
+        <v/>
+      </c>
+      <c r="E13">
+        <f>ROUND((C13-D13)*$B$7,2)</f>
+        <v/>
+      </c>
+      <c r="F13">
+        <f>C13-D13-E13</f>
+        <v/>
+      </c>
+      <c r="G13">
+        <f>F13/C13</f>
+        <v/>
+      </c>
+      <c r="H13" s="2" t="n">
+        <v>0.12</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Avg ticket (40% sedan / 40% SUV / 20% truck)</t>
-        </is>
-      </c>
-      <c r="B14">
-        <f>0.4*B10+0.4*B11+0.2*B12</f>
-        <v/>
+          <t>Luxury</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>SUV</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="n">
+        <v>379</v>
+      </c>
+      <c r="D14">
+        <f>$B$6</f>
+        <v/>
+      </c>
+      <c r="E14">
+        <f>ROUND((C14-D14)*$B$7,2)</f>
+        <v/>
+      </c>
+      <c r="F14">
+        <f>C14-D14-E14</f>
+        <v/>
+      </c>
+      <c r="G14">
+        <f>F14/C14</f>
+        <v/>
+      </c>
+      <c r="H14" s="2" t="n">
+        <v>0.12</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Avg Morgan keeps per job: subcontractors</t>
-        </is>
-      </c>
-      <c r="B15">
-        <f>0.4*E10+0.4*E11+0.2*E12</f>
-        <v/>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>Avg Morgan keeps per job: tech pay</t>
-        </is>
-      </c>
-      <c r="B16">
-        <f>0.4*I10+0.4*I11+0.2*I12</f>
+          <t>Luxury</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Truck / 3-row</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="n">
+        <v>399</v>
+      </c>
+      <c r="D15">
+        <f>$B$6</f>
+        <v/>
+      </c>
+      <c r="E15">
+        <f>ROUND((C15-D15)*$B$7,2)</f>
+        <v/>
+      </c>
+      <c r="F15">
+        <f>C15-D15-E15</f>
+        <v/>
+      </c>
+      <c r="G15">
+        <f>F15/C15</f>
+        <v/>
+      </c>
+      <c r="H15" s="2" t="n">
+        <v>0.06</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Average ticket (by job mix)</t>
+        </is>
+      </c>
+      <c r="B17">
+        <f>SUMPRODUCT(C10:C15,H10:H15)</f>
         <v/>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="1" t="inlineStr">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Average you keep per job</t>
+        </is>
+      </c>
+      <c r="B18">
+        <f>SUMPRODUCT(F10:F15,H10:H15)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="1" t="inlineStr">
         <is>
           <t>Monthly revenue</t>
         </is>
       </c>
-      <c r="B18" t="inlineStr">
+      <c r="B20" t="inlineStr">
         <is>
           <t>Jobs</t>
         </is>
       </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>Morgan keeps (subcontractors)</t>
-        </is>
-      </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>Morgan keeps (tech pay)</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="n">
-        <v>10000</v>
-      </c>
-      <c r="B19">
-        <f>ROUNDUP(A19/$B$14,0)</f>
-        <v/>
-      </c>
-      <c r="C19">
-        <f>ROUND(B19*$B$15,0)</f>
-        <v/>
-      </c>
-      <c r="D19">
-        <f>ROUND(B19*$B$16,0)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="n">
-        <v>20000</v>
-      </c>
-      <c r="B20">
-        <f>ROUNDUP(A20/$B$14,0)</f>
-        <v/>
-      </c>
-      <c r="C20">
-        <f>ROUND(B20*$B$15,0)</f>
-        <v/>
-      </c>
-      <c r="D20">
-        <f>ROUND(B20*$B$16,0)</f>
-        <v/>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>You keep</t>
+        </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
-        <v>30000</v>
+        <v>10000</v>
       </c>
       <c r="B21">
-        <f>ROUNDUP(A21/$B$14,0)</f>
+        <f>ROUNDUP(A21/$B$17,0)</f>
         <v/>
       </c>
       <c r="C21">
-        <f>ROUND(B21*$B$15,0)</f>
-        <v/>
-      </c>
-      <c r="D21">
-        <f>ROUND(B21*$B$16,0)</f>
+        <f>ROUND(B21*$B$18,0)</f>
         <v/>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="n">
-        <v>50000</v>
+        <v>20000</v>
       </c>
       <c r="B22">
-        <f>ROUNDUP(A22/$B$14,0)</f>
+        <f>ROUNDUP(A22/$B$17,0)</f>
         <v/>
       </c>
       <c r="C22">
-        <f>ROUND(B22*$B$15,0)</f>
-        <v/>
-      </c>
-      <c r="D22">
-        <f>ROUND(B22*$B$16,0)</f>
+        <f>ROUND(B22*$B$18,0)</f>
         <v/>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="n">
+        <v>30000</v>
+      </c>
+      <c r="B23">
+        <f>ROUNDUP(A23/$B$17,0)</f>
+        <v/>
+      </c>
+      <c r="C23">
+        <f>ROUND(B23*$B$18,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>50000</v>
+      </c>
+      <c r="B24">
+        <f>ROUNDUP(A24/$B$17,0)</f>
+        <v/>
+      </c>
+      <c r="C24">
+        <f>ROUND(B24*$B$18,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
         <v>100000</v>
       </c>
-      <c r="B23">
-        <f>ROUNDUP(A23/$B$14,0)</f>
-        <v/>
-      </c>
-      <c r="C23">
-        <f>ROUND(B23*$B$15,0)</f>
-        <v/>
-      </c>
-      <c r="D23">
-        <f>ROUND(B23*$B$16,0)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="1" t="inlineStr">
-        <is>
-          <t>ADD-ONS (no Rapid Reach fee; get a yes before starting)</t>
-        </is>
-      </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>Price</t>
-        </is>
-      </c>
-      <c r="C25" t="inlineStr">
-        <is>
-          <t>Sub (60%)</t>
-        </is>
-      </c>
-      <c r="D25" t="inlineStr">
-        <is>
-          <t>Morgan (40%)</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>Pet hair removal</t>
-        </is>
-      </c>
-      <c r="B26" t="n">
-        <v>50</v>
-      </c>
-      <c r="C26">
-        <f>B26*$B$7</f>
-        <v/>
-      </c>
-      <c r="D26">
-        <f>B26*(1-$B$7)</f>
+      <c r="B25">
+        <f>ROUNDUP(A25/$B$17,0)</f>
+        <v/>
+      </c>
+      <c r="C25">
+        <f>ROUND(B25*$B$18,0)</f>
         <v/>
       </c>
     </row>
     <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>Heavy pet hair</t>
-        </is>
-      </c>
-      <c r="B27" t="n">
-        <v>100</v>
-      </c>
-      <c r="C27">
-        <f>B27*$B$7</f>
-        <v/>
-      </c>
-      <c r="D27">
-        <f>B27*(1-$B$7)</f>
-        <v/>
+      <c r="A27" s="1" t="inlineStr">
+        <is>
+          <t>WHAT'S INCLUDED</t>
+        </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Seat / stain extraction (per seat)</t>
-        </is>
-      </c>
-      <c r="B28" t="n">
-        <v>40</v>
-      </c>
-      <c r="C28">
-        <f>B28*$B$7</f>
-        <v/>
-      </c>
-      <c r="D28">
-        <f>B28*(1-$B$7)</f>
-        <v/>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Inside: full vacuum (seats, carpets, trunk), seats and carpets spot-treated, dash, console, doors and vents cleaned and protected, door jambs, inside windows, floor mats. Outside: hand wash, wheels, tires and wheel wells, tire shine, bug and tar removal, windows, spray sealant.</t>
+        </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Carpet + mat shampoo</t>
-        </is>
-      </c>
-      <c r="B29" t="n">
-        <v>75</v>
-      </c>
-      <c r="C29">
-        <f>B29*$B$7</f>
-        <v/>
-      </c>
-      <c r="D29">
-        <f>B29*(1-$B$7)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>Odor removal (ozone)</t>
-        </is>
-      </c>
-      <c r="B30" t="n">
-        <v>75</v>
-      </c>
-      <c r="C30">
-        <f>B30*$B$7</f>
-        <v/>
-      </c>
-      <c r="D30">
-        <f>B30*(1-$B$7)</f>
-        <v/>
+          <t>Luxury</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Everything in Standard, plus deep shampoo of all seats, carpets and floor mats; leather cleaned and conditioned; hand wax buffed to a deep shine (1–2 months protection); trim restored; engine bay cleaned.</t>
+        </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t>Headlight restoration</t>
-        </is>
-      </c>
-      <c r="B31" t="n">
-        <v>75</v>
-      </c>
-      <c r="C31">
-        <f>B31*$B$7</f>
-        <v/>
-      </c>
-      <c r="D31">
-        <f>B31*(1-$B$7)</f>
-        <v/>
+      <c r="A31" s="1" t="inlineStr">
+        <is>
+          <t>ADD-ONS (no Rapid Reach fee; get a yes before starting)</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Price</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Sub (60%)</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>You (40%)</t>
+        </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Engine bay clean</t>
+          <t>Pet hair removal</t>
         </is>
       </c>
       <c r="B32" t="n">
@@ -945,11 +907,11 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Clay bar + paint sealant (6 months)</t>
+          <t>Heavy pet hair</t>
         </is>
       </c>
       <c r="B33" t="n">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="C33">
         <f>B33*$B$7</f>
@@ -963,11 +925,11 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Heavy dirt / sand / mud</t>
+          <t>Odor removal (ozone)</t>
         </is>
       </c>
       <c r="B34" t="n">
-        <v>50</v>
+        <v>75</v>
       </c>
       <c r="C34">
         <f>B34*$B$7</f>
@@ -981,11 +943,11 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Biohazard (from)</t>
+          <t>Headlight restoration</t>
         </is>
       </c>
       <c r="B35" t="n">
-        <v>150</v>
+        <v>75</v>
       </c>
       <c r="C35">
         <f>B35*$B$7</f>
@@ -999,11 +961,11 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Travel (45+ min)</t>
+          <t>Clay bar + paint sealant (6 months)</t>
         </is>
       </c>
       <c r="B36" t="n">
-        <v>35</v>
+        <v>99</v>
       </c>
       <c r="C36">
         <f>B36*$B$7</f>
@@ -1014,52 +976,92 @@
         <v/>
       </c>
     </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Heavy dirt / sand / mud</t>
+        </is>
+      </c>
+      <c r="B37" t="n">
+        <v>50</v>
+      </c>
+      <c r="C37">
+        <f>B37*$B$7</f>
+        <v/>
+      </c>
+      <c r="D37">
+        <f>B37*(1-$B$7)</f>
+        <v/>
+      </c>
+    </row>
     <row r="38">
-      <c r="A38" s="1" t="inlineStr">
-        <is>
-          <t>PRICE RULES</t>
-        </is>
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Biohazard (from)</t>
+        </is>
+      </c>
+      <c r="B38" t="n">
+        <v>150</v>
+      </c>
+      <c r="C38">
+        <f>B38*$B$7</f>
+        <v/>
+      </c>
+      <c r="D38">
+        <f>B38*(1-$B$7)</f>
+        <v/>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Full Detail only: Sedan $234, SUV $285, Truck $325. No packages.</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" t="inlineStr">
-        <is>
-          <t>Always ask the year, make and model before quoting.</t>
-        </is>
+          <t>Travel (45+ min)</t>
+        </is>
+      </c>
+      <c r="B39" t="n">
+        <v>35</v>
+      </c>
+      <c r="C39">
+        <f>B39*$B$7</f>
+        <v/>
+      </c>
+      <c r="D39">
+        <f>B39*(1-$B$7)</f>
+        <v/>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>On the call: mention pet hair / stains / smell add-on prices if the customer brings them up.</t>
+          <t>PRICE RULES</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>On site: walk around with the customer, point out what you see, quote the add-on from this list, get a yes (text is fine) BEFORE starting.</t>
+          <t>Two packages only: Standard and Luxury. Pitch Luxury first, step down to Standard.</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Never add a charge after the job. Never invent prices on the spot; only use this list.</t>
+          <t>Always ask the year, make and model before quoting.</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Tech pay model: Morgan buys supplies. Subcontractor model: subs pay their own chemicals and gas.</t>
+          <t>Never go below Standard. If they can't afford it, offer to keep them on the list for a special.</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>Add-ons: walk around the car, quote from this list, get a yes BEFORE starting. Never charge after the job.</t>
         </is>
       </c>
     </row>

</xml_diff>